<commit_message>
fix(workspace-web): 重點速覽 placeholder 縮短避免 textarea 裁切
範例句移至欄位下方 hint 完整顯示；Naive UI textarea placeholder
為 overflow hidden 疊層，autosize 高度不含 placeholder 導致多行被裁。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/workspace-web/i18n.xlsx
+++ b/apps/workspace-web/i18n.xlsx
@@ -5449,21 +5449,19 @@
     <t>legalDocs.highlightsPlaceholder</t>
   </si>
   <si>
-    <t xml:space="preserve">每行一則，以第一個「|」分隔標題與描述，例如：
-作品永遠是你的|上架不會轉移著作權，創作者僅授權平台展示與銷售作品。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One per line, title and description split by the first "|", e.g.:
-Your work stays yours|Listing never transfers copyright — creators only license us to display and sell their work.</t>
+    <t>每行一則，格式：標題|描述</t>
+  </si>
+  <si>
+    <t>One per line, format: title|description</t>
   </si>
   <si>
     <t>legalDocs.highlightsHint</t>
   </si>
   <si>
-    <t>選填，最多 6 則；顯示於前台條款頁頂部的 30 秒摘要卡，留空則前台改用預設文案。</t>
-  </si>
-  <si>
-    <t>Optional, up to 6 items; shown as the 30-second summary cards atop the public legal page. Leave empty to fall back to the default copy.</t>
+    <t>選填，最多 6 則；顯示於前台條款頁頂部的 30 秒摘要卡，留空則前台改用預設文案。例如：作品永遠是你的|上架不會轉移著作權，創作者僅授權平台展示與銷售作品。</t>
+  </si>
+  <si>
+    <t>Optional, up to 6 items; shown as the 30-second summary cards atop the public legal page. Leave empty to fall back to the default copy. E.g.: Your work stays yours|Listing never transfers copyright — creators only license us to display and sell their work.</t>
   </si>
   <si>
     <t>legalDocs.valHighlightsFormat</t>

</xml_diff>